<commit_message>
fix some of bugggs
</commit_message>
<xml_diff>
--- a/public/quick submittion-template.xlsx
+++ b/public/quick submittion-template.xlsx
@@ -5,18 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TOSHIBA\Desktop\val system\ValueTech-Frontend\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TOSHIBA\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA1C12DF-305D-472A-A739-1CDDF4D3C674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1437377F-F4CA-4B1F-8302-645D62724D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="market" sheetId="2" r:id="rId1"/>
     <sheet name="cost" sheetId="3" r:id="rId2"/>
     <sheet name="data" sheetId="4" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="UsageList">data!$F$3:$F$21</definedName>
+  </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1716" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1756" uniqueCount="177">
   <si>
     <t>purpose_id</t>
   </si>
@@ -1656,12 +1659,41 @@
   <si>
     <t>تحديد</t>
   </si>
+  <si>
+    <t xml:space="preserve">مياه
+</t>
+  </si>
+  <si>
+    <t>asset1</t>
+  </si>
+  <si>
+    <t>asset2</t>
+  </si>
+  <si>
+    <t>asset3</t>
+  </si>
+  <si>
+    <t>asset4</t>
+  </si>
+  <si>
+    <t>asset5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">بناء
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">منطقة الرياض </t>
+  </si>
+  <si>
+    <t xml:space="preserve">الرياض </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1690,6 +1722,11 @@
       <color theme="1"/>
       <name val="arial"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Noto Sans Arabic UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1744,7 +1781,63 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Noto Sans Arabic UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1755,6 +1848,17 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0074DED1-B9D8-4C63-8666-B12D189A001F}" name="Table1" displayName="Table1" ref="E1:F21" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="E1:F21" xr:uid="{0074DED1-B9D8-4C63-8666-B12D189A001F}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{D948C097-1600-46AE-97CE-B7B1F4167382}" name="code" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{2D422985-F57F-430A-8ADD-FA987EEAF8CD}" name="Asset Being Valued Usage\Sector" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2012,13 +2116,27 @@
       <c r="AC1" s="2"/>
     </row>
     <row r="2" spans="1:29" ht="15.75">
-      <c r="A2" s="1"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D2" s="5">
+        <v>1000</v>
+      </c>
+      <c r="E2" s="12">
+        <v>46022</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="H2" s="7"/>
       <c r="I2" s="1"/>
       <c r="J2" s="2"/>
@@ -2040,13 +2158,27 @@
       <c r="Z2" s="8"/>
     </row>
     <row r="3" spans="1:29" ht="15.75">
-      <c r="A3" s="1"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1100</v>
+      </c>
+      <c r="E3" s="12">
+        <v>46023</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="H3" s="7"/>
       <c r="I3" s="1"/>
       <c r="J3" s="2"/>
@@ -2065,13 +2197,27 @@
       <c r="W3" s="2"/>
     </row>
     <row r="4" spans="1:29" ht="15.75">
-      <c r="A4" s="1"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1200</v>
+      </c>
+      <c r="E4" s="12">
+        <v>46055</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="H4" s="7"/>
       <c r="I4" s="1"/>
       <c r="J4" s="2"/>
@@ -2090,13 +2236,27 @@
       <c r="W4" s="2"/>
     </row>
     <row r="5" spans="1:29" ht="15.75">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1300</v>
+      </c>
+      <c r="E5" s="12">
+        <v>46040</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -2113,13 +2273,27 @@
       <c r="W5" s="2"/>
     </row>
     <row r="6" spans="1:29" ht="15.75">
-      <c r="A6" s="1"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1400</v>
+      </c>
+      <c r="E6" s="12">
+        <v>46058</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -2158,7 +2332,8 @@
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
     </row>
-    <row r="8" spans="1:29">
+    <row r="8" spans="1:29" ht="15.75">
+      <c r="C8" s="1"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="J8" s="2"/>
@@ -2176,7 +2351,8 @@
       <c r="V8" s="2"/>
       <c r="W8" s="2"/>
     </row>
-    <row r="9" spans="1:29">
+    <row r="9" spans="1:29" ht="15.75">
+      <c r="C9" s="1"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="J9" s="2"/>
@@ -2194,7 +2370,8 @@
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
     </row>
-    <row r="10" spans="1:29">
+    <row r="10" spans="1:29" ht="15.75">
+      <c r="C10" s="1"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
       <c r="J10" s="2"/>
@@ -2212,7 +2389,8 @@
       <c r="V10" s="2"/>
       <c r="W10" s="2"/>
     </row>
-    <row r="11" spans="1:29">
+    <row r="11" spans="1:29" ht="15.75">
+      <c r="C11" s="1"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
       <c r="J11" s="2"/>
@@ -2230,7 +2408,8 @@
       <c r="V11" s="2"/>
       <c r="W11" s="2"/>
     </row>
-    <row r="12" spans="1:29">
+    <row r="12" spans="1:29" ht="15.75">
+      <c r="C12" s="1"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="J12" s="2"/>
@@ -2248,7 +2427,8 @@
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
     </row>
-    <row r="13" spans="1:29">
+    <row r="13" spans="1:29" ht="15.75">
+      <c r="C13" s="1"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="J13" s="2"/>
@@ -2266,7 +2446,8 @@
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
     </row>
-    <row r="14" spans="1:29">
+    <row r="14" spans="1:29" ht="15.75">
+      <c r="C14" s="1"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="J14" s="2"/>
@@ -2284,7 +2465,8 @@
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
     </row>
-    <row r="15" spans="1:29">
+    <row r="15" spans="1:29" ht="15.75">
+      <c r="C15" s="1"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="J15" s="2"/>
@@ -2302,7 +2484,8 @@
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
     </row>
-    <row r="16" spans="1:29">
+    <row r="16" spans="1:29" ht="15.75">
+      <c r="C16" s="1"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="J16" s="2"/>
@@ -2320,7 +2503,8 @@
       <c r="V16" s="2"/>
       <c r="W16" s="2"/>
     </row>
-    <row r="17" spans="4:23">
+    <row r="17" spans="3:23" ht="15.75">
+      <c r="C17" s="1"/>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="J17" s="2"/>
@@ -2338,7 +2522,8 @@
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
     </row>
-    <row r="18" spans="4:23">
+    <row r="18" spans="3:23" ht="15.75">
+      <c r="C18" s="1"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="J18" s="2"/>
@@ -2356,7 +2541,8 @@
       <c r="V18" s="2"/>
       <c r="W18" s="2"/>
     </row>
-    <row r="19" spans="4:23">
+    <row r="19" spans="3:23" ht="15.75">
+      <c r="C19" s="1"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="J19" s="2"/>
@@ -2374,7 +2560,8 @@
       <c r="V19" s="2"/>
       <c r="W19" s="2"/>
     </row>
-    <row r="20" spans="4:23">
+    <row r="20" spans="3:23" ht="15.75">
+      <c r="C20" s="1"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
       <c r="J20" s="2"/>
@@ -2392,7 +2579,8 @@
       <c r="V20" s="2"/>
       <c r="W20" s="2"/>
     </row>
-    <row r="21" spans="4:23" ht="15.75" customHeight="1">
+    <row r="21" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C21" s="1"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="J21" s="2"/>
@@ -2410,7 +2598,8 @@
       <c r="V21" s="2"/>
       <c r="W21" s="2"/>
     </row>
-    <row r="22" spans="4:23" ht="15.75" customHeight="1">
+    <row r="22" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C22" s="1"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
       <c r="J22" s="2"/>
@@ -2428,7 +2617,8 @@
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
     </row>
-    <row r="23" spans="4:23" ht="15.75" customHeight="1">
+    <row r="23" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C23" s="1"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
       <c r="J23" s="2"/>
@@ -2446,7 +2636,8 @@
       <c r="V23" s="2"/>
       <c r="W23" s="2"/>
     </row>
-    <row r="24" spans="4:23" ht="15.75" customHeight="1">
+    <row r="24" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C24" s="1"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
       <c r="J24" s="2"/>
@@ -2464,7 +2655,8 @@
       <c r="V24" s="2"/>
       <c r="W24" s="2"/>
     </row>
-    <row r="25" spans="4:23" ht="15.75" customHeight="1">
+    <row r="25" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C25" s="1"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
       <c r="J25" s="2"/>
@@ -2482,7 +2674,8 @@
       <c r="V25" s="2"/>
       <c r="W25" s="2"/>
     </row>
-    <row r="26" spans="4:23" ht="15.75" customHeight="1">
+    <row r="26" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C26" s="1"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
       <c r="J26" s="2"/>
@@ -2500,7 +2693,8 @@
       <c r="V26" s="2"/>
       <c r="W26" s="2"/>
     </row>
-    <row r="27" spans="4:23" ht="15.75" customHeight="1">
+    <row r="27" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C27" s="1"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
       <c r="J27" s="2"/>
@@ -2518,7 +2712,8 @@
       <c r="V27" s="2"/>
       <c r="W27" s="2"/>
     </row>
-    <row r="28" spans="4:23" ht="15.75" customHeight="1">
+    <row r="28" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C28" s="1"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
       <c r="J28" s="2"/>
@@ -2536,7 +2731,8 @@
       <c r="V28" s="2"/>
       <c r="W28" s="2"/>
     </row>
-    <row r="29" spans="4:23" ht="15.75" customHeight="1">
+    <row r="29" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C29" s="1"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
       <c r="J29" s="2"/>
@@ -2554,7 +2750,8 @@
       <c r="V29" s="2"/>
       <c r="W29" s="2"/>
     </row>
-    <row r="30" spans="4:23" ht="15.75" customHeight="1">
+    <row r="30" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C30" s="1"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
       <c r="J30" s="2"/>
@@ -2572,7 +2769,8 @@
       <c r="V30" s="2"/>
       <c r="W30" s="2"/>
     </row>
-    <row r="31" spans="4:23" ht="15.75" customHeight="1">
+    <row r="31" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C31" s="1"/>
       <c r="D31" s="5"/>
       <c r="E31" s="5"/>
       <c r="J31" s="2"/>
@@ -2590,7 +2788,8 @@
       <c r="V31" s="2"/>
       <c r="W31" s="2"/>
     </row>
-    <row r="32" spans="4:23" ht="15.75" customHeight="1">
+    <row r="32" spans="3:23" ht="15.75" customHeight="1">
+      <c r="C32" s="1"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
       <c r="J32" s="2"/>
@@ -18473,6 +18672,12 @@
       <c r="W1000" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{AC1EEE43-B146-426D-AFC6-935F5333017E}">
+      <formula1>UsageList</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <extLst>
@@ -18570,13 +18775,27 @@
       <c r="AC1" s="2"/>
     </row>
     <row r="2" spans="1:29" ht="15.75">
-      <c r="A2" s="1"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2" s="5">
+        <v>1000</v>
+      </c>
+      <c r="E2" s="12">
+        <v>46022</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="H2" s="7"/>
       <c r="I2" s="1"/>
       <c r="J2" s="2"/>
@@ -18598,13 +18817,27 @@
       <c r="Z2" s="8"/>
     </row>
     <row r="3" spans="1:29" ht="15.75">
-      <c r="A3" s="1"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1100</v>
+      </c>
+      <c r="E3" s="12">
+        <v>46023</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="H3" s="7"/>
       <c r="I3" s="1"/>
       <c r="J3" s="2"/>
@@ -18623,13 +18856,27 @@
       <c r="W3" s="2"/>
     </row>
     <row r="4" spans="1:29" ht="15.75">
-      <c r="A4" s="1"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1200</v>
+      </c>
+      <c r="E4" s="12">
+        <v>46055</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="H4" s="7"/>
       <c r="I4" s="1"/>
       <c r="J4" s="2"/>
@@ -18648,22 +18895,50 @@
       <c r="W4" s="2"/>
     </row>
     <row r="5" spans="1:29" ht="15.75">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1300</v>
+      </c>
+      <c r="E5" s="12">
+        <v>46040</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="6" spans="1:29" ht="15.75">
-      <c r="A6" s="1"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1400</v>
+      </c>
+      <c r="E6" s="12">
+        <v>46058</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="7" spans="1:29" ht="15.75">
       <c r="A7" s="1"/>
@@ -21829,6 +22104,11 @@
       <c r="C1000" s="2"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{CA0F26A7-0758-4C54-9BE6-8C5135E01419}">
+      <formula1>UsageList</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <extLst>
@@ -21859,7 +22139,7 @@
     <col min="3" max="3" width="8.109375" customWidth="1"/>
     <col min="4" max="4" width="18.109375" customWidth="1"/>
     <col min="5" max="5" width="11.5546875" customWidth="1"/>
-    <col min="6" max="6" width="14.77734375" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" customWidth="1"/>
     <col min="7" max="7" width="12.44140625" customWidth="1"/>
     <col min="8" max="8" width="4.5546875" customWidth="1"/>
     <col min="9" max="9" width="11" customWidth="1"/>
@@ -22008,7 +22288,7 @@
         <v>4210000088</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="61.5">
+    <row r="5" spans="1:11" ht="31.5">
       <c r="A5" s="1">
         <v>5</v>
       </c>
@@ -22078,7 +22358,7 @@
         <v>4210000091</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="46.5">
+    <row r="7" spans="1:11" ht="31.5">
       <c r="A7" s="1">
         <v>8</v>
       </c>
@@ -22142,7 +22422,7 @@
         <v>4210000375</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="46.5">
+    <row r="9" spans="1:11" ht="31.5">
       <c r="A9" s="1">
         <v>10</v>
       </c>
@@ -30488,5 +30768,8 @@
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>